<commit_message>
Update menu visibility and prices
</commit_message>
<xml_diff>
--- a/deliverables/bedri-usta-webmenu-version-138-tr-de-en.xlsx
+++ b/deliverables/bedri-usta-webmenu-version-138-tr-de-en.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Türkçe" sheetId="1" r:id="Re9a8a3c18e63461f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deutsch" sheetId="2" r:id="Ra645150f0919446e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="English" sheetId="3" r:id="R63ff8bc7686c4421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Türkçe" sheetId="1" r:id="R7be0dba599684ac0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deutsch" sheetId="2" r:id="Rd37e1ff3475149a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="English" sheetId="3" r:id="Ra34ecf331c914bb1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4387,7 +4387,7 @@
         <x:v>Adana - Tavuk Şiş</x:v>
       </x:c>
       <x:c r="E113" s="4" t="n">
-        <x:v>18.9</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="F113" s="3" t="str">
         <x:v>Adana kebap, tavuk şiş, domates, sivri biber, patates kızartması veya pilav ile</x:v>
@@ -4422,7 +4422,7 @@
         <x:v>Adana - Kuzu Şiş</x:v>
       </x:c>
       <x:c r="E114" s="4" t="n">
-        <x:v>19.9</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="F114" s="3" t="str">
         <x:v>Adana kebap, kuzu şiş, domates, sivri biber, patates kızartması veya pilav ile</x:v>
@@ -4457,7 +4457,7 @@
         <x:v>Kuzu Şiş - Tavuk Şiş</x:v>
       </x:c>
       <x:c r="E115" s="4" t="n">
-        <x:v>19.9</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="F115" s="3" t="str">
         <x:v>Kuzu eti, marine tavuk, domates, sivri biber, patates kızartması veya pilav ile</x:v>
@@ -5647,7 +5647,7 @@
         <x:v>Yaprak Dürüm</x:v>
       </x:c>
       <x:c r="E149" s="4" t="n">
-        <x:v>9.9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F149" s="3" t="str">
         <x:v>Yaprak döner, taze garnitürler, lavaş</x:v>
@@ -5682,7 +5682,7 @@
         <x:v>Yaprak Ekmek Arası</x:v>
       </x:c>
       <x:c r="E150" s="4" t="n">
-        <x:v>8.9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F150" s="3" t="str">
         <x:v>Yaprak döner, taze garnitürler, ekmek</x:v>
@@ -5717,7 +5717,7 @@
         <x:v>Yaprak Döner Menü</x:v>
       </x:c>
       <x:c r="E151" s="4" t="n">
-        <x:v>12.9</x:v>
+        <x:v>18.9</x:v>
       </x:c>
       <x:c r="F151" s="3" t="str">
         <x:v>Yaprak döner, pilav veya patates seçimi</x:v>
@@ -5787,7 +5787,7 @@
         <x:v>İskender</x:v>
       </x:c>
       <x:c r="E153" s="4" t="n">
-        <x:v>16.9</x:v>
+        <x:v>19.9</x:v>
       </x:c>
       <x:c r="F153" s="3" t="str">
         <x:v>Yaprak döner, iskender sosu, yoğurt</x:v>
@@ -16198,7 +16198,7 @@
         <x:v>Adana &amp; Hähnchenspieß</x:v>
       </x:c>
       <x:c r="F113" s="4" t="n">
-        <x:v>18.9</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="G113" s="3" t="str">
         <x:v>Adana Kebap, Hähnchenspieß, Tomate, Peperoni, mit Pommes frites oder Reis</x:v>
@@ -16236,7 +16236,7 @@
         <x:v>Adana &amp; Lammspieß</x:v>
       </x:c>
       <x:c r="F114" s="4" t="n">
-        <x:v>19.9</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="G114" s="3" t="str">
         <x:v>Adana Kebap, Lammspieß, Tomate, Peperoni, mit Pommes frites oder Reis</x:v>
@@ -16274,7 +16274,7 @@
         <x:v>Lamm- &amp; Hähnchenspieß</x:v>
       </x:c>
       <x:c r="F115" s="4" t="n">
-        <x:v>19.9</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="G115" s="3" t="str">
         <x:v>Lammfleisch, mariniertes Hähnchen, Tomate, Peperoni, mit Pommes frites oder Reis</x:v>
@@ -17566,7 +17566,7 @@
         <x:v>Döner-Wrap</x:v>
       </x:c>
       <x:c r="F149" s="4" t="n">
-        <x:v>9.9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G149" s="3" t="str">
         <x:v>Yaprak-Döner, frische Garnitur, Lavash</x:v>
@@ -17604,7 +17604,7 @@
         <x:v>Döner im Brot</x:v>
       </x:c>
       <x:c r="F150" s="4" t="n">
-        <x:v>8.9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G150" s="3" t="str">
         <x:v>Yaprak-Döner, frische Garnitur, Brot</x:v>
@@ -17642,7 +17642,7 @@
         <x:v>Döner-Menü</x:v>
       </x:c>
       <x:c r="F151" s="4" t="n">
-        <x:v>12.9</x:v>
+        <x:v>18.9</x:v>
       </x:c>
       <x:c r="G151" s="3" t="str">
         <x:v>Yaprak-Döner, Reis oder Pommes frites nach Wahl</x:v>
@@ -17718,7 +17718,7 @@
         <x:v>Iskender Kebap</x:v>
       </x:c>
       <x:c r="F153" s="4" t="n">
-        <x:v>16.9</x:v>
+        <x:v>19.9</x:v>
       </x:c>
       <x:c r="G153" s="3" t="str">
         <x:v>Yaprak-Döner, Iskender-Sauce, Joghurt</x:v>
@@ -28549,7 +28549,7 @@
         <x:v>Adana &amp; Chicken Skewer</x:v>
       </x:c>
       <x:c r="F113" s="4" t="n">
-        <x:v>18.9</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="G113" s="3" t="str">
         <x:v>Adana kebap, chicken skewer, tomato, long green pepper, with French fries or rice</x:v>
@@ -28587,7 +28587,7 @@
         <x:v>Adana &amp; Lamb Skewer</x:v>
       </x:c>
       <x:c r="F114" s="4" t="n">
-        <x:v>19.9</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="G114" s="3" t="str">
         <x:v>Adana kebap, lamb skewer, tomato, long green pepper, with French fries or rice</x:v>
@@ -28625,7 +28625,7 @@
         <x:v>Lamb &amp; Chicken Skewer</x:v>
       </x:c>
       <x:c r="F115" s="4" t="n">
-        <x:v>19.9</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="G115" s="3" t="str">
         <x:v>Lamb, marinated chicken, tomato, long green pepper, with French fries or rice</x:v>
@@ -29917,7 +29917,7 @@
         <x:v>Döner Wrap</x:v>
       </x:c>
       <x:c r="F149" s="4" t="n">
-        <x:v>9.9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G149" s="3" t="str">
         <x:v>Yaprak döner, fresh garnish, lavash</x:v>
@@ -29955,7 +29955,7 @@
         <x:v>Döner in Bread</x:v>
       </x:c>
       <x:c r="F150" s="4" t="n">
-        <x:v>8.9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G150" s="3" t="str">
         <x:v>Yaprak döner, fresh garnish, bread</x:v>
@@ -29993,7 +29993,7 @@
         <x:v>Döner Menu</x:v>
       </x:c>
       <x:c r="F151" s="4" t="n">
-        <x:v>12.9</x:v>
+        <x:v>18.9</x:v>
       </x:c>
       <x:c r="G151" s="3" t="str">
         <x:v>Yaprak döner, rice or French fries of your choice</x:v>
@@ -30069,7 +30069,7 @@
         <x:v>Iskender Kebap</x:v>
       </x:c>
       <x:c r="F153" s="4" t="n">
-        <x:v>16.9</x:v>
+        <x:v>19.9</x:v>
       </x:c>
       <x:c r="G153" s="3" t="str">
         <x:v>Yaprak döner, Iskender sauce, yoghurt</x:v>

</xml_diff>